<commit_message>
chuc_nang(import_nguyenvong): them chuc nang import list nguyen vong day
</commit_message>
<xml_diff>
--- a/1_data_excel/Nguyện_vọng_dạy_của_giảng_viên.xlsx
+++ b/1_data_excel/Nguyện_vọng_dạy_của_giảng_viên.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\.PROJECT_1\1_data_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45C594A9-3DEF-46DF-8F37-0D6920579F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A049159-3FE4-4791-B7B3-04D73AD60A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="158">
   <si>
     <t>Tên học phần</t>
   </si>
@@ -486,6 +486,15 @@
   </si>
   <si>
     <t>Lê Văn Phong - DN01701267; Trần Hải Anh - DN01801851; Đỗ Thị Huyền - DN01801855; Lê Thái Bảo - DN01801850</t>
+  </si>
+  <si>
+    <t>Hệ thống máy tính lượng tử</t>
+  </si>
+  <si>
+    <t>FAKE01</t>
+  </si>
+  <si>
+    <t>Nguyễn Lượng Tử - DN0999999</t>
   </si>
 </sst>
 </file>
@@ -1733,9 +1742,19 @@
         <v>153</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" spans="1:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B64" t="s">
+        <v>156</v>
+      </c>
+      <c r="C64" t="s">
+        <v>157</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C13:C1048576 C1:C11">
+  <conditionalFormatting sqref="C1:C11 C13:C1048576">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Trần Vũ Đại"</formula>
     </cfRule>

</xml_diff>